<commit_message>
Renamed Sheets & Added one
</commit_message>
<xml_diff>
--- a/B&B Multi Sheet Workbook.xlsx
+++ b/B&B Multi Sheet Workbook.xlsx
@@ -1,34 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adame\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Excel Beginner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{19D53418-C581-4964-94C1-F16F8F0B4CC4}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{242B3EDE-EF0D-44B7-AD72-5A43A6DFBFF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
-    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
-    <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
-    <sheet name="Sheet6" sheetId="6" r:id="rId6"/>
-    <sheet name="Sheet7" sheetId="7" r:id="rId7"/>
-    <sheet name="Sheet8" sheetId="8" r:id="rId8"/>
-    <sheet name="Sheet9" sheetId="9" r:id="rId9"/>
-    <sheet name="Sheet10" sheetId="10" r:id="rId10"/>
-    <sheet name="Sheet11" sheetId="11" r:id="rId11"/>
-    <sheet name="Sheet12" sheetId="12" r:id="rId12"/>
-    <sheet name="Sheet13" sheetId="13" r:id="rId13"/>
-    <sheet name="Sheet14" sheetId="14" r:id="rId14"/>
-    <sheet name="Sheet15" sheetId="15" r:id="rId15"/>
-    <sheet name="Sheet16" sheetId="16" r:id="rId16"/>
+    <sheet name="Australia" sheetId="1" r:id="rId1"/>
+    <sheet name="Europe" sheetId="2" r:id="rId2"/>
+    <sheet name="N America" sheetId="3" r:id="rId3"/>
+    <sheet name="S America" sheetId="4" r:id="rId4"/>
+    <sheet name="Summary" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="17" r:id="rId6"/>
+    <sheet name="Sheet6" sheetId="6" r:id="rId7"/>
+    <sheet name="Sheet7" sheetId="7" r:id="rId8"/>
+    <sheet name="Sheet8" sheetId="8" r:id="rId9"/>
+    <sheet name="Sheet9" sheetId="9" r:id="rId10"/>
+    <sheet name="Sheet10" sheetId="10" r:id="rId11"/>
+    <sheet name="Sheet11" sheetId="11" r:id="rId12"/>
+    <sheet name="Sheet12" sheetId="12" r:id="rId13"/>
+    <sheet name="Sheet13" sheetId="13" r:id="rId14"/>
+    <sheet name="Sheet14" sheetId="14" r:id="rId15"/>
+    <sheet name="Sheet15" sheetId="15" r:id="rId16"/>
+    <sheet name="Sheet16" sheetId="16" r:id="rId17"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -95,8 +96,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -143,7 +144,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -153,7 +154,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -538,17 +539,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.33203125" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -565,7 +566,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -582,7 +583,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -599,7 +600,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -616,7 +617,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -633,7 +634,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>10</v>
       </c>
@@ -665,9 +666,23 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <phoneticPr fontId="0" type="halfwidthKatakana" alignment="noControl"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter alignWithMargins="0">
+    <oddHeader>&amp;A</oddHeader>
+    <oddFooter>Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="0" type="halfwidthKatakana" alignment="noControl"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -678,10 +693,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="0" type="halfwidthKatakana" alignment="noControl"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -692,10 +707,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="0" type="halfwidthKatakana" alignment="noControl"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -706,10 +721,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="0" type="halfwidthKatakana" alignment="noControl"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -720,10 +735,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="0" type="halfwidthKatakana" alignment="noControl"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -734,10 +749,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="0" type="halfwidthKatakana" alignment="noControl"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -748,10 +763,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="0" type="halfwidthKatakana" alignment="noControl"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -765,22 +780,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.33203125" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -797,7 +812,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -814,7 +829,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -831,7 +846,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -848,7 +863,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -865,7 +880,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>10</v>
       </c>
@@ -899,17 +914,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.33203125" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -926,7 +941,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -943,7 +958,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -960,7 +975,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -977,7 +992,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -994,7 +1009,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>10</v>
       </c>
@@ -1028,17 +1043,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.33203125" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -1055,7 +1070,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1072,7 +1087,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -1089,7 +1104,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1106,7 +1121,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1123,7 +1138,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>10</v>
       </c>
@@ -1157,17 +1172,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.33203125" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -1184,27 +1199,27 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>10</v>
       </c>
@@ -1236,9 +1251,18 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94F6FD81-4CF2-4E81-85B6-E2618ED1D549}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="0" type="halfwidthKatakana" alignment="noControl"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1249,10 +1273,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="0" type="halfwidthKatakana" alignment="noControl"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1263,10 +1287,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="0" type="halfwidthKatakana" alignment="noControl"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1275,18 +1299,4 @@
     <oddFooter>Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <phoneticPr fontId="0" type="halfwidthKatakana" alignment="noControl"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter alignWithMargins="0">
-    <oddHeader>&amp;A</oddHeader>
-    <oddFooter>Page &amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>